<commit_message>
Merge switch ctrl,RTC timing update
</commit_message>
<xml_diff>
--- a/Pin_Define/STM32F103C8_Pin_Define.xlsx
+++ b/Pin_Define/STM32F103C8_Pin_Define.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My Embedded\My_test_Prj\a\MQTT_Selserver_GameRoom\Pin_Define\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C9B40AE-C8CA-4F8D-8B56-563A8B8F09F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95714B82-B015-4455-A195-0E19C50381CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10780" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,9 +84,6 @@
     <t>PC14</t>
   </si>
   <si>
-    <t>OSC32_IN</t>
-  </si>
-  <si>
     <t>PC15-OSC32_OUT</t>
   </si>
   <si>
@@ -232,9 +229,6 @@
   </si>
   <si>
     <t>TIM4</t>
-  </si>
-  <si>
-    <t>按下开关后门磁计时关断，时钟每次计时1s</t>
   </si>
   <si>
     <t xml:space="preserve">PB10 </t>
@@ -525,6 +519,14 @@
   </si>
   <si>
     <t>增加心跳检测30s</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>按下开关后门磁计时关断，时钟每次计时1s</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSC32_IN</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -532,7 +534,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -593,6 +595,13 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="12">
@@ -729,7 +738,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -787,6 +796,27 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -796,12 +826,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -811,9 +835,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -823,19 +844,10 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1130,15 +1142,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1217,8 +1229,8 @@
       <c r="E5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>17</v>
+      <c r="F5" s="36" t="s">
+        <v>161</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5"/>
@@ -1231,17 +1243,17 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>19</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>20</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6"/>
@@ -1254,14 +1266,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>22</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
@@ -1275,14 +1287,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
@@ -1296,14 +1308,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
@@ -1317,14 +1329,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -1338,14 +1350,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
@@ -1359,47 +1371,47 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="7"/>
+      <c r="H12" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="22"/>
-      <c r="O12" s="22"/>
-      <c r="P12" s="22"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="21"/>
+      <c r="P12" s="21"/>
     </row>
     <row r="13" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13"/>
@@ -1412,23 +1424,23 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="G14" s="7"/>
-      <c r="H14" s="27" t="s">
-        <v>71</v>
-      </c>
-      <c r="I14" s="27"/>
+      <c r="H14" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="24"/>
       <c r="J14"/>
       <c r="K14"/>
     </row>
@@ -1437,23 +1449,23 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="G15" s="7"/>
-      <c r="H15" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="I15" s="23"/>
+      <c r="H15" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="I15" s="25"/>
       <c r="J15"/>
       <c r="K15"/>
     </row>
@@ -1462,17 +1474,17 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16"/>
@@ -1485,17 +1497,17 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17"/>
@@ -1508,58 +1520,58 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>49</v>
       </c>
       <c r="H18"/>
       <c r="I18"/>
       <c r="J18"/>
-      <c r="K18" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-      <c r="N18" s="32"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="32"/>
+      <c r="K18" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>17</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="G19" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="H19"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
@@ -1572,29 +1584,29 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="G20" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="H20"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="L20" s="35" t="s">
-        <v>161</v>
+        <v>57</v>
+      </c>
+      <c r="L20" s="19" t="s">
+        <v>159</v>
       </c>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -1606,26 +1618,26 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>61</v>
       </c>
       <c r="H21"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
@@ -1638,16 +1650,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="E22" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>65</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -1655,12 +1667,12 @@
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="L22" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="M22" s="34"/>
+        <v>65</v>
+      </c>
+      <c r="L22" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="M22" s="23"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
@@ -1670,26 +1682,26 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="J23"/>
       <c r="K23" s="17" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
@@ -1702,26 +1714,26 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="J24"/>
       <c r="K24" s="17" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
@@ -1734,14 +1746,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
@@ -1760,14 +1772,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
@@ -1786,23 +1798,23 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F27" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E27" s="6" t="s">
+      <c r="G27" s="7"/>
+      <c r="H27" s="30" t="s">
         <v>81</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="G27" s="7"/>
-      <c r="H27" s="25" t="s">
-        <v>83</v>
       </c>
       <c r="I27"/>
       <c r="J27"/>
@@ -1818,22 +1830,22 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G28" s="7"/>
-      <c r="H28" s="25"/>
+      <c r="H28" s="30"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28" s="13"/>
@@ -1848,22 +1860,22 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G29" s="7"/>
-      <c r="H29" s="25"/>
+      <c r="H29" s="30"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29" s="13"/>
@@ -1878,22 +1890,22 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G30" s="7"/>
-      <c r="H30" s="25"/>
+      <c r="H30" s="30"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -1903,60 +1915,60 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="G31" s="7"/>
       <c r="H31"/>
       <c r="I31"/>
       <c r="J31"/>
-      <c r="K31" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="L31" s="20"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="20"/>
-      <c r="O31" s="20"/>
-      <c r="P31" s="21"/>
+      <c r="K31" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="L31" s="27"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
+      <c r="P31" s="28"/>
     </row>
     <row r="32" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6">
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G32" s="7"/>
-      <c r="H32" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="I32" s="27"/>
+      <c r="H32" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="I32" s="24"/>
       <c r="J32"/>
       <c r="K32" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15"/>
@@ -1969,28 +1981,28 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G33" s="7"/>
-      <c r="H33" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="I33" s="23"/>
+      <c r="H33" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="I33" s="25"/>
       <c r="J33"/>
       <c r="K33" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15"/>
@@ -2003,26 +2015,26 @@
         <v>32</v>
       </c>
       <c r="B34" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>102</v>
       </c>
       <c r="G34" s="7"/>
       <c r="H34"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34" s="14" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15"/>
@@ -2035,52 +2047,52 @@
         <v>33</v>
       </c>
       <c r="B35" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F35" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="G35" s="7"/>
-      <c r="H35" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="22"/>
-      <c r="M35" s="22"/>
-      <c r="N35" s="22"/>
-      <c r="O35" s="22"/>
-      <c r="P35" s="22"/>
+      <c r="H35" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+      <c r="M35" s="21"/>
+      <c r="N35" s="21"/>
+      <c r="O35" s="21"/>
+      <c r="P35" s="21"/>
     </row>
     <row r="36" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="8">
         <v>34</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>12</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H36"/>
       <c r="I36"/>
@@ -2092,14 +2104,14 @@
         <v>35</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
@@ -2113,14 +2125,14 @@
         <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
@@ -2134,20 +2146,20 @@
         <v>37</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>12</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H39"/>
       <c r="I39"/>
@@ -2159,26 +2171,26 @@
         <v>38</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F40" s="7"/>
       <c r="G40" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="H40" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="I40" t="s">
         <v>119</v>
-      </c>
-      <c r="H40" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="I40" t="s">
-        <v>121</v>
       </c>
       <c r="J40"/>
       <c r="K40"/>
@@ -2193,22 +2205,22 @@
         <v>39</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F41" s="7"/>
       <c r="G41" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="H41" s="25"/>
+        <v>122</v>
+      </c>
+      <c r="H41" s="30"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
@@ -2218,22 +2230,22 @@
         <v>40</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F42" s="7"/>
       <c r="G42" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="H42" s="25"/>
+        <v>125</v>
+      </c>
+      <c r="H42" s="30"/>
       <c r="I42"/>
       <c r="J42"/>
       <c r="K42"/>
@@ -2243,27 +2255,27 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G43" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="H43" s="18" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="I43" s="16"/>
-      <c r="J43" s="29" t="s">
-        <v>155</v>
+      <c r="J43" s="33" t="s">
+        <v>153</v>
       </c>
       <c r="K43"/>
     </row>
@@ -2272,28 +2284,28 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G44" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C44" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="H44" s="18" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I44" s="16"/>
-      <c r="J44" s="30"/>
+      <c r="J44" s="34"/>
       <c r="K44"/>
     </row>
     <row r="45" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2301,28 +2313,28 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="G45" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C45" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>136</v>
-      </c>
       <c r="H45" s="18" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I45" s="16"/>
-      <c r="J45" s="30"/>
+      <c r="J45" s="34"/>
       <c r="K45"/>
     </row>
     <row r="46" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2330,14 +2342,14 @@
         <v>44</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2351,29 +2363,29 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="G47" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C47" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="F47" s="6" t="s">
+      <c r="H47" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="G47" s="6" t="s">
+      <c r="I47" s="25"/>
+      <c r="J47" t="s">
         <v>141</v>
-      </c>
-      <c r="H47" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="I47" s="23"/>
-      <c r="J47" t="s">
-        <v>143</v>
       </c>
       <c r="K47"/>
     </row>
@@ -2382,29 +2394,29 @@
         <v>46</v>
       </c>
       <c r="B48" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G48" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C48" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="F48" s="6" t="s">
+      <c r="H48" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="I48" s="29"/>
+      <c r="J48" t="s">
         <v>146</v>
-      </c>
-      <c r="H48" s="24" t="s">
-        <v>147</v>
-      </c>
-      <c r="I48" s="24"/>
-      <c r="J48" t="s">
-        <v>148</v>
       </c>
       <c r="K48"/>
     </row>
@@ -2413,14 +2425,14 @@
         <v>47</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
@@ -2430,26 +2442,20 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D50" s="4"/>
       <c r="E50" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H12:P12"/>
-    <mergeCell ref="K18:P18"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
     <mergeCell ref="K31:P31"/>
     <mergeCell ref="H35:P35"/>
     <mergeCell ref="H47:I47"/>
@@ -2459,6 +2465,12 @@
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="J43:J45"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H12:P12"/>
+    <mergeCell ref="K18:P18"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lamp and door delay,add voice
</commit_message>
<xml_diff>
--- a/Pin_Define/STM32F103C8_Pin_Define.xlsx
+++ b/Pin_Define/STM32F103C8_Pin_Define.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My Embedded\My_test_Prj\a\MQTT_Selserver_GameRoom\Pin_Define\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95714B82-B015-4455-A195-0E19C50381CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AC6E5D-5B14-41EA-86F1-8108C6C51782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10780" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="176">
   <si>
     <t>STM32F103C8T6引脚定义表</t>
   </si>
@@ -518,15 +518,71 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>增加心跳检测30s</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>按下开关后门磁计时关断，时钟每次计时1s</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>OSC32_IN</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ESP12F-EN</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ESP12F-RST</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>W25Q64</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q64-SCK</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q64-MISO</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q64-MOSI</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q64-CS</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>JR6001_RX</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>JR6001_TX</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ReadPin_BUSY</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Relay_1_Pin_DoorLock</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Relay_2_Pin_Light</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Relay_3_Pin_AllSocket</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Relay_4_Pin_else</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>增加心跳检测定时</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -534,7 +590,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -603,8 +659,17 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -671,8 +736,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -732,13 +815,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -799,6 +900,18 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -808,6 +921,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -817,6 +933,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -844,10 +963,31 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1129,30 +1269,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P50"/>
-  <sheetFormatPr defaultColWidth="16.58203125" defaultRowHeight="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="16.625" defaultRowHeight="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.375" style="1" customWidth="1"/>
     <col min="2" max="2" width="21.25" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.375" style="1" customWidth="1"/>
     <col min="5" max="5" width="14.25" style="1" customWidth="1"/>
-    <col min="6" max="6" width="46.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="46.875" style="1" customWidth="1"/>
     <col min="7" max="7" width="37.25" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="16.58203125" style="1"/>
+    <col min="8" max="16384" width="16.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-    </row>
-    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+    </row>
+    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1175,7 +1315,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1192,7 +1332,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>2</v>
       </c>
@@ -1215,7 +1355,7 @@
       <c r="J4"/>
       <c r="K4"/>
     </row>
-    <row r="5" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -1229,8 +1369,8 @@
       <c r="E5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="36" t="s">
-        <v>161</v>
+      <c r="F5" s="20" t="s">
+        <v>160</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5"/>
@@ -1238,7 +1378,7 @@
       <c r="J5"/>
       <c r="K5"/>
     </row>
-    <row r="6" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>4</v>
       </c>
@@ -1261,7 +1401,7 @@
       <c r="J6"/>
       <c r="K6"/>
     </row>
-    <row r="7" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1282,7 +1422,7 @@
       <c r="J7"/>
       <c r="K7"/>
     </row>
-    <row r="8" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -1303,7 +1443,7 @@
       <c r="J8"/>
       <c r="K8"/>
     </row>
-    <row r="9" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -1324,7 +1464,7 @@
       <c r="J9"/>
       <c r="K9"/>
     </row>
-    <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -1345,7 +1485,7 @@
       <c r="J10"/>
       <c r="K10"/>
     </row>
-    <row r="11" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -1366,7 +1506,7 @@
       <c r="J11"/>
       <c r="K11"/>
     </row>
-    <row r="12" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>10</v>
       </c>
@@ -1384,19 +1524,19 @@
         <v>34</v>
       </c>
       <c r="G12" s="7"/>
-      <c r="H12" s="21" t="s">
+      <c r="H12" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
-      <c r="L12" s="21"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="21"/>
-      <c r="O12" s="21"/>
-      <c r="P12" s="21"/>
-    </row>
-    <row r="13" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="25"/>
+      <c r="N12" s="25"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="25"/>
+    </row>
+    <row r="13" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>11</v>
       </c>
@@ -1419,7 +1559,7 @@
       <c r="J13"/>
       <c r="K13"/>
     </row>
-    <row r="14" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>12</v>
       </c>
@@ -1437,14 +1577,14 @@
         <v>39</v>
       </c>
       <c r="G14" s="7"/>
-      <c r="H14" s="24" t="s">
+      <c r="H14" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="I14" s="24"/>
+      <c r="I14" s="29"/>
       <c r="J14"/>
       <c r="K14"/>
     </row>
-    <row r="15" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>13</v>
       </c>
@@ -1462,14 +1602,14 @@
         <v>41</v>
       </c>
       <c r="G15" s="7"/>
-      <c r="H15" s="25" t="s">
+      <c r="H15" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="I15" s="25"/>
+      <c r="I15" s="30"/>
       <c r="J15"/>
       <c r="K15"/>
     </row>
-    <row r="16" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>14</v>
       </c>
@@ -1487,12 +1627,16 @@
         <v>43</v>
       </c>
       <c r="G16" s="7"/>
-      <c r="H16"/>
-      <c r="I16"/>
+      <c r="H16" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="I16" s="22" t="s">
+        <v>167</v>
+      </c>
       <c r="J16"/>
       <c r="K16"/>
     </row>
-    <row r="17" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>15</v>
       </c>
@@ -1510,12 +1654,14 @@
         <v>45</v>
       </c>
       <c r="G17" s="7"/>
-      <c r="H17"/>
-      <c r="I17"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="22" t="s">
+        <v>164</v>
+      </c>
       <c r="J17"/>
       <c r="K17"/>
     </row>
-    <row r="18" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>16</v>
       </c>
@@ -1535,19 +1681,21 @@
       <c r="G18" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H18"/>
-      <c r="I18"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="21" t="s">
+        <v>165</v>
+      </c>
       <c r="J18"/>
-      <c r="K18" s="22" t="s">
+      <c r="K18" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="22"/>
-    </row>
-    <row r="19" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
+    </row>
+    <row r="19" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>17</v>
       </c>
@@ -1567,8 +1715,10 @@
       <c r="G19" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H19"/>
-      <c r="I19"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="21" t="s">
+        <v>166</v>
+      </c>
       <c r="J19"/>
       <c r="K19" s="12" t="s">
         <v>53</v>
@@ -1579,7 +1729,7 @@
       <c r="O19" s="11"/>
       <c r="P19" s="11"/>
     </row>
-    <row r="20" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>18</v>
       </c>
@@ -1606,14 +1756,14 @@
         <v>57</v>
       </c>
       <c r="L20" s="19" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
       <c r="O20" s="11"/>
       <c r="P20" s="11"/>
     </row>
-    <row r="21" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>19</v>
       </c>
@@ -1645,7 +1795,7 @@
       <c r="O21" s="11"/>
       <c r="P21" s="11"/>
     </row>
-    <row r="22" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>20</v>
       </c>
@@ -1669,15 +1819,15 @@
       <c r="K22" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="L22" s="35" t="s">
-        <v>160</v>
-      </c>
-      <c r="M22" s="23"/>
+      <c r="L22" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="M22" s="28"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
     </row>
-    <row r="23" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>21</v>
       </c>
@@ -1699,6 +1849,10 @@
       <c r="G23" s="6" t="s">
         <v>68</v>
       </c>
+      <c r="H23" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="I23" s="45"/>
       <c r="J23"/>
       <c r="K23" s="17" t="s">
         <v>154</v>
@@ -1709,7 +1863,7 @@
       <c r="O23" s="11"/>
       <c r="P23" s="11"/>
     </row>
-    <row r="24" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>22</v>
       </c>
@@ -1730,6 +1884,12 @@
       </c>
       <c r="G24" s="6" t="s">
         <v>72</v>
+      </c>
+      <c r="H24" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="I24" s="44" t="s">
+        <v>170</v>
       </c>
       <c r="J24"/>
       <c r="K24" s="17" t="s">
@@ -1741,7 +1901,7 @@
       <c r="O24" s="11"/>
       <c r="P24" s="11"/>
     </row>
-    <row r="25" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>23</v>
       </c>
@@ -1757,7 +1917,6 @@
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25" s="13"/>
@@ -1767,7 +1926,7 @@
       <c r="O25" s="11"/>
       <c r="P25" s="11"/>
     </row>
-    <row r="26" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>24</v>
       </c>
@@ -1793,7 +1952,7 @@
       <c r="O26" s="11"/>
       <c r="P26" s="11"/>
     </row>
-    <row r="27" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>25</v>
       </c>
@@ -1813,11 +1972,13 @@
         <v>80</v>
       </c>
       <c r="G27" s="7"/>
-      <c r="H27" s="30" t="s">
+      <c r="H27" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="I27"/>
-      <c r="J27"/>
+      <c r="I27" s="46" t="s">
+        <v>171</v>
+      </c>
+      <c r="J27" s="47"/>
       <c r="K27" s="13"/>
       <c r="L27" s="11"/>
       <c r="M27" s="11"/>
@@ -1825,7 +1986,7 @@
       <c r="O27" s="11"/>
       <c r="P27" s="11"/>
     </row>
-    <row r="28" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>26</v>
       </c>
@@ -1845,9 +2006,11 @@
         <v>83</v>
       </c>
       <c r="G28" s="7"/>
-      <c r="H28" s="30"/>
-      <c r="I28"/>
-      <c r="J28"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="49" t="s">
+        <v>172</v>
+      </c>
+      <c r="J28" s="48"/>
       <c r="K28" s="13"/>
       <c r="L28" s="11"/>
       <c r="M28" s="11"/>
@@ -1855,7 +2018,7 @@
       <c r="O28" s="11"/>
       <c r="P28" s="11"/>
     </row>
-    <row r="29" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
         <v>27</v>
       </c>
@@ -1875,9 +2038,11 @@
         <v>85</v>
       </c>
       <c r="G29" s="7"/>
-      <c r="H29" s="30"/>
-      <c r="I29"/>
-      <c r="J29"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="49" t="s">
+        <v>173</v>
+      </c>
+      <c r="J29" s="48"/>
       <c r="K29" s="13"/>
       <c r="L29" s="11"/>
       <c r="M29" s="11"/>
@@ -1885,7 +2050,7 @@
       <c r="O29" s="11"/>
       <c r="P29" s="11"/>
     </row>
-    <row r="30" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="6">
         <v>28</v>
       </c>
@@ -1905,12 +2070,14 @@
         <v>87</v>
       </c>
       <c r="G30" s="7"/>
-      <c r="H30" s="30"/>
-      <c r="I30"/>
-      <c r="J30"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="49" t="s">
+        <v>174</v>
+      </c>
+      <c r="J30" s="36"/>
       <c r="K30"/>
     </row>
-    <row r="31" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="6">
         <v>29</v>
       </c>
@@ -1933,16 +2100,16 @@
       <c r="H31"/>
       <c r="I31"/>
       <c r="J31"/>
-      <c r="K31" s="26" t="s">
+      <c r="K31" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="L31" s="27"/>
-      <c r="M31" s="27"/>
-      <c r="N31" s="27"/>
-      <c r="O31" s="27"/>
-      <c r="P31" s="28"/>
-    </row>
-    <row r="32" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+      <c r="P31" s="34"/>
+    </row>
+    <row r="32" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
         <v>30</v>
       </c>
@@ -1962,10 +2129,10 @@
         <v>93</v>
       </c>
       <c r="G32" s="7"/>
-      <c r="H32" s="31" t="s">
+      <c r="H32" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="I32" s="24"/>
+      <c r="I32" s="29"/>
       <c r="J32"/>
       <c r="K32" s="14" t="s">
         <v>94</v>
@@ -1976,7 +2143,7 @@
       <c r="O32" s="15"/>
       <c r="P32" s="15"/>
     </row>
-    <row r="33" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
         <v>31</v>
       </c>
@@ -1996,10 +2163,10 @@
         <v>96</v>
       </c>
       <c r="G33" s="7"/>
-      <c r="H33" s="32" t="s">
+      <c r="H33" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="I33" s="25"/>
+      <c r="I33" s="30"/>
       <c r="J33"/>
       <c r="K33" s="14" t="s">
         <v>97</v>
@@ -2010,7 +2177,7 @@
       <c r="O33" s="15"/>
       <c r="P33" s="15"/>
     </row>
-    <row r="34" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
         <v>32</v>
       </c>
@@ -2042,7 +2209,7 @@
       <c r="O34" s="15"/>
       <c r="P34" s="15"/>
     </row>
-    <row r="35" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>33</v>
       </c>
@@ -2062,19 +2229,19 @@
         <v>104</v>
       </c>
       <c r="G35" s="7"/>
-      <c r="H35" s="21" t="s">
+      <c r="H35" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="21"/>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="21"/>
-      <c r="O35" s="21"/>
-      <c r="P35" s="21"/>
-    </row>
-    <row r="36" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I35" s="25"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+    </row>
+    <row r="36" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
         <v>34</v>
       </c>
@@ -2099,7 +2266,7 @@
       <c r="J36"/>
       <c r="K36"/>
     </row>
-    <row r="37" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>35</v>
       </c>
@@ -2120,7 +2287,7 @@
       <c r="J37"/>
       <c r="K37"/>
     </row>
-    <row r="38" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>36</v>
       </c>
@@ -2141,7 +2308,7 @@
       <c r="J38"/>
       <c r="K38"/>
     </row>
-    <row r="39" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="8">
         <v>37</v>
       </c>
@@ -2166,7 +2333,7 @@
       <c r="J39"/>
       <c r="K39"/>
     </row>
-    <row r="40" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="6">
         <v>38</v>
       </c>
@@ -2186,7 +2353,7 @@
       <c r="G40" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="H40" s="30" t="s">
+      <c r="H40" s="36" t="s">
         <v>118</v>
       </c>
       <c r="I40" t="s">
@@ -2200,7 +2367,7 @@
       <c r="O40"/>
       <c r="P40"/>
     </row>
-    <row r="41" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>39</v>
       </c>
@@ -2220,12 +2387,12 @@
       <c r="G41" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H41" s="30"/>
+      <c r="H41" s="36"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
     </row>
-    <row r="42" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <v>40</v>
       </c>
@@ -2245,12 +2412,12 @@
       <c r="G42" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H42" s="30"/>
+      <c r="H42" s="36"/>
       <c r="I42"/>
       <c r="J42"/>
       <c r="K42"/>
     </row>
-    <row r="43" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
         <v>41</v>
       </c>
@@ -2274,12 +2441,12 @@
         <v>156</v>
       </c>
       <c r="I43" s="16"/>
-      <c r="J43" s="33" t="s">
+      <c r="J43" s="39" t="s">
         <v>153</v>
       </c>
       <c r="K43"/>
     </row>
-    <row r="44" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
         <v>42</v>
       </c>
@@ -2305,10 +2472,10 @@
         <v>157</v>
       </c>
       <c r="I44" s="16"/>
-      <c r="J44" s="34"/>
+      <c r="J44" s="40"/>
       <c r="K44"/>
     </row>
-    <row r="45" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>43</v>
       </c>
@@ -2334,10 +2501,10 @@
         <v>158</v>
       </c>
       <c r="I45" s="16"/>
-      <c r="J45" s="34"/>
+      <c r="J45" s="40"/>
       <c r="K45"/>
     </row>
-    <row r="46" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="8">
         <v>44</v>
       </c>
@@ -2358,7 +2525,7 @@
       <c r="J46"/>
       <c r="K46"/>
     </row>
-    <row r="47" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6">
         <v>45</v>
       </c>
@@ -2380,16 +2547,20 @@
       <c r="G47" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H47" s="25" t="s">
+      <c r="H47" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="I47" s="25"/>
+      <c r="I47" s="30"/>
       <c r="J47" t="s">
         <v>141</v>
       </c>
       <c r="K47"/>
-    </row>
-    <row r="48" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L47" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="M47" s="42"/>
+    </row>
+    <row r="48" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6">
         <v>46</v>
       </c>
@@ -2411,16 +2582,20 @@
       <c r="G48" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="H48" s="29" t="s">
+      <c r="H48" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="I48" s="29"/>
+      <c r="I48" s="35"/>
       <c r="J48" t="s">
         <v>146</v>
       </c>
       <c r="K48"/>
-    </row>
-    <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L48" s="43" t="s">
+        <v>162</v>
+      </c>
+      <c r="M48" s="35"/>
+    </row>
+    <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>47</v>
       </c>
@@ -2437,7 +2612,7 @@
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
     </row>
-    <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4">
         <v>48</v>
       </c>
@@ -2455,7 +2630,7 @@
       <c r="G50" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="22">
     <mergeCell ref="K31:P31"/>
     <mergeCell ref="H35:P35"/>
     <mergeCell ref="H47:I47"/>
@@ -2465,12 +2640,19 @@
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="J43:J45"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J30"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="H12:P12"/>
     <mergeCell ref="K18:P18"/>
     <mergeCell ref="L22:M22"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H16:H19"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add flash store and JR6001 sound
</commit_message>
<xml_diff>
--- a/Pin_Define/STM32F103C8_Pin_Define.xlsx
+++ b/Pin_Define/STM32F103C8_Pin_Define.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My Embedded\My_test_Prj\a\MQTT_Selserver_GameRoom\Pin_Define\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AC6E5D-5B14-41EA-86F1-8108C6C51782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF3D624-5C3B-4AC2-80BD-4F1539E285CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="373" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -744,13 +745,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="8" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -839,7 +840,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -903,21 +904,75 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -927,67 +982,25 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1282,15 +1295,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -1524,17 +1537,17 @@
         <v>34</v>
       </c>
       <c r="G12" s="7"/>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
     </row>
     <row r="13" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
@@ -1577,10 +1590,10 @@
         <v>39</v>
       </c>
       <c r="G14" s="7"/>
-      <c r="H14" s="29" t="s">
+      <c r="H14" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="I14" s="29"/>
+      <c r="I14" s="32"/>
       <c r="J14"/>
       <c r="K14"/>
     </row>
@@ -1602,124 +1615,124 @@
         <v>41</v>
       </c>
       <c r="G15" s="7"/>
-      <c r="H15" s="30" t="s">
+      <c r="H15" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="I15" s="30"/>
+      <c r="I15" s="28"/>
       <c r="J15"/>
       <c r="K15"/>
     </row>
     <row r="16" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="6">
+      <c r="A16" s="47">
         <v>14</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6" t="s">
+      <c r="C16" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="G16" s="7"/>
-      <c r="H16" s="31" t="s">
+      <c r="G16" s="49"/>
+      <c r="H16" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="I16" s="22" t="s">
+      <c r="I16" s="51" t="s">
         <v>167</v>
       </c>
-      <c r="J16"/>
+      <c r="J16" s="52"/>
       <c r="K16"/>
     </row>
     <row r="17" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6">
+      <c r="A17" s="47">
         <v>15</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
+      <c r="C17" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="G17" s="7"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="22" t="s">
+      <c r="G17" s="49"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="J17"/>
+      <c r="J17" s="52"/>
       <c r="K17"/>
     </row>
     <row r="18" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="6">
+      <c r="A18" s="47">
         <v>16</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
+      <c r="C18" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="H18" s="31"/>
-      <c r="I18" s="21" t="s">
+      <c r="H18" s="50"/>
+      <c r="I18" s="53" t="s">
         <v>165</v>
       </c>
-      <c r="J18"/>
-      <c r="K18" s="26" t="s">
+      <c r="J18" s="52"/>
+      <c r="K18" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="44"/>
+      <c r="N18" s="44"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
     </row>
     <row r="19" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="6">
+      <c r="A19" s="47">
         <v>17</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6" t="s">
+      <c r="C19" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="47" t="s">
         <v>52</v>
       </c>
-      <c r="H19" s="31"/>
-      <c r="I19" s="21" t="s">
+      <c r="H19" s="50"/>
+      <c r="I19" s="53" t="s">
         <v>166</v>
       </c>
-      <c r="J19"/>
+      <c r="J19" s="52"/>
       <c r="K19" s="12" t="s">
         <v>53</v>
       </c>
@@ -1819,10 +1832,10 @@
       <c r="K22" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="L22" s="27" t="s">
+      <c r="L22" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M22" s="28"/>
+      <c r="M22" s="46"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
@@ -1849,10 +1862,10 @@
       <c r="G23" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="I23" s="45"/>
+      <c r="I23" s="23"/>
       <c r="J23"/>
       <c r="K23" s="17" t="s">
         <v>154</v>
@@ -1885,10 +1898,10 @@
       <c r="G24" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="45" t="s">
+      <c r="H24" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="I24" s="44" t="s">
+      <c r="I24" s="22" t="s">
         <v>170</v>
       </c>
       <c r="J24"/>
@@ -1972,13 +1985,13 @@
         <v>80</v>
       </c>
       <c r="G27" s="7"/>
-      <c r="H27" s="36" t="s">
+      <c r="H27" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="I27" s="46" t="s">
+      <c r="I27" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="J27" s="47"/>
+      <c r="J27" s="40"/>
       <c r="K27" s="13"/>
       <c r="L27" s="11"/>
       <c r="M27" s="11"/>
@@ -2006,11 +2019,11 @@
         <v>83</v>
       </c>
       <c r="G28" s="7"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="49" t="s">
+      <c r="H28" s="30"/>
+      <c r="I28" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="J28" s="48"/>
+      <c r="J28" s="42"/>
       <c r="K28" s="13"/>
       <c r="L28" s="11"/>
       <c r="M28" s="11"/>
@@ -2038,11 +2051,11 @@
         <v>85</v>
       </c>
       <c r="G29" s="7"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="49" t="s">
+      <c r="H29" s="30"/>
+      <c r="I29" s="41" t="s">
         <v>173</v>
       </c>
-      <c r="J29" s="48"/>
+      <c r="J29" s="42"/>
       <c r="K29" s="13"/>
       <c r="L29" s="11"/>
       <c r="M29" s="11"/>
@@ -2070,11 +2083,11 @@
         <v>87</v>
       </c>
       <c r="G30" s="7"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="49" t="s">
+      <c r="H30" s="30"/>
+      <c r="I30" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J30" s="36"/>
+      <c r="J30" s="30"/>
       <c r="K30"/>
     </row>
     <row r="31" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2100,14 +2113,14 @@
       <c r="H31"/>
       <c r="I31"/>
       <c r="J31"/>
-      <c r="K31" s="32" t="s">
+      <c r="K31" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-      <c r="O31" s="33"/>
-      <c r="P31" s="34"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
+      <c r="N31" s="25"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="26"/>
     </row>
     <row r="32" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
@@ -2129,10 +2142,10 @@
         <v>93</v>
       </c>
       <c r="G32" s="7"/>
-      <c r="H32" s="37" t="s">
+      <c r="H32" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="I32" s="29"/>
+      <c r="I32" s="32"/>
       <c r="J32"/>
       <c r="K32" s="14" t="s">
         <v>94</v>
@@ -2163,10 +2176,10 @@
         <v>96</v>
       </c>
       <c r="G33" s="7"/>
-      <c r="H33" s="38" t="s">
+      <c r="H33" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="I33" s="30"/>
+      <c r="I33" s="28"/>
       <c r="J33"/>
       <c r="K33" s="14" t="s">
         <v>97</v>
@@ -2229,17 +2242,17 @@
         <v>104</v>
       </c>
       <c r="G35" s="7"/>
-      <c r="H35" s="25" t="s">
+      <c r="H35" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="I35" s="25"/>
-      <c r="J35" s="25"/>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="25"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="27"/>
+      <c r="M35" s="27"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
     </row>
     <row r="36" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
@@ -2353,7 +2366,7 @@
       <c r="G40" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="H40" s="36" t="s">
+      <c r="H40" s="30" t="s">
         <v>118</v>
       </c>
       <c r="I40" t="s">
@@ -2387,7 +2400,7 @@
       <c r="G41" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H41" s="36"/>
+      <c r="H41" s="30"/>
       <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
@@ -2412,7 +2425,7 @@
       <c r="G42" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="H42" s="36"/>
+      <c r="H42" s="30"/>
       <c r="I42"/>
       <c r="J42"/>
       <c r="K42"/>
@@ -2441,7 +2454,7 @@
         <v>156</v>
       </c>
       <c r="I43" s="16"/>
-      <c r="J43" s="39" t="s">
+      <c r="J43" s="34" t="s">
         <v>153</v>
       </c>
       <c r="K43"/>
@@ -2472,7 +2485,7 @@
         <v>157</v>
       </c>
       <c r="I44" s="16"/>
-      <c r="J44" s="40"/>
+      <c r="J44" s="35"/>
       <c r="K44"/>
     </row>
     <row r="45" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2501,7 +2514,7 @@
         <v>158</v>
       </c>
       <c r="I45" s="16"/>
-      <c r="J45" s="40"/>
+      <c r="J45" s="35"/>
       <c r="K45"/>
     </row>
     <row r="46" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2547,18 +2560,18 @@
       <c r="G47" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H47" s="30" t="s">
+      <c r="H47" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="I47" s="30"/>
+      <c r="I47" s="28"/>
       <c r="J47" t="s">
         <v>141</v>
       </c>
       <c r="K47"/>
-      <c r="L47" s="41" t="s">
+      <c r="L47" s="36" t="s">
         <v>161</v>
       </c>
-      <c r="M47" s="42"/>
+      <c r="M47" s="37"/>
     </row>
     <row r="48" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6">
@@ -2582,18 +2595,18 @@
       <c r="G48" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="H48" s="35" t="s">
+      <c r="H48" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="I48" s="35"/>
+      <c r="I48" s="29"/>
       <c r="J48" t="s">
         <v>146</v>
       </c>
       <c r="K48"/>
-      <c r="L48" s="43" t="s">
+      <c r="L48" s="38" t="s">
         <v>162</v>
       </c>
-      <c r="M48" s="35"/>
+      <c r="M48" s="29"/>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
@@ -2631,6 +2644,13 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H12:P12"/>
+    <mergeCell ref="K18:P18"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="H16:H19"/>
     <mergeCell ref="K31:P31"/>
     <mergeCell ref="H35:P35"/>
     <mergeCell ref="H47:I47"/>
@@ -2646,13 +2666,6 @@
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="I29:J29"/>
     <mergeCell ref="I30:J30"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H12:P12"/>
-    <mergeCell ref="K18:P18"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H16:H19"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>